<commit_message>
COSMoS behavioural analysis: align documents and reference files
- New root-level SDTM_Domain_Overview.md: three analytical layers (CT, domain, COSMoS)
- Behavioural_Group column added to Domain_Analysis.xlsx and Pattern_Inventory.xlsx
- Content_and_QC.md: IS target-driven fix, actual QC values, cross-refs
- README.md: mermaid data flow, COSMoS docs visible
- Remove old Domain_Overview from sdtm-domain-reference/docs/
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/reports/SDTM_Domain_Analysis.xlsx
+++ b/sdtm-domain-reference/reports/SDTM_Domain_Analysis.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +111,12 @@
         <fgColor rgb="00D6DCE4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -204,6 +214,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B114"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -578,753 +595,625 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>SDTM Domain Analysis</t>
+        </is>
+      </c>
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PROVENANCE</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Base data</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SDTM_Domain_Metadata.xlsx (this track, machine_actionable/)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>CT analysis</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>sdtm-ct-analysis skill — 1,181 codelists, 25 categories</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>COSMoS data</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>COSMoS_BC_DSS.xlsx from cosmos-bc-dss track</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/kerfors/cdisc-for-ai</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>INPUTS</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>The Structural_Type categorization is derived from two analytical inputs:</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1. SDTM CT Category Discovery</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Assignments</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>skills/sdtm-ct-analysis/example-output/SDTM_CT_Category_Discovery_assignments.csv</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Profiles</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>skills/sdtm-ct-analysis/example-output/SDTM_CT_Category_Profiles.md</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Key finding</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>25 categories; 83% of codelists (976/1181) are instrument-specific;</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>extensibility flag separates 56 domain-level from 353 instrument-specific test code codelists</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
+      <c r="A18" s="2" t="inlineStr"/>
       <c r="B18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2. COSMoS BC/DSS content analysis</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Interim file</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cosmos-bc-dss/interim/COSMoS_BC_DSS.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Content doc</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>cosmos-bc-dss/docs/COSMoS_Content_and_QC.md</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Key finding</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BC-&gt;DSS decomposition by specimen/method only occurs in specimen-based domains;</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-    </row>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>instrument domains are 1:1 (DSS=BC); BC hierarchy provides instrument-&gt;question grouping</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>3. COSMoS Behavioural Analysis</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Analysis doc</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>cosmos-bc-dss/docs/COSMoS_Behavioural_Analysis.md</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Reference file</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>cosmos-bc-dss/docs/COSMoS_Domain_Pattern_Inventory.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Key finding</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>10 behavioural groups; Specimen-based splits into 3 distinct patterns; 6 decomposition axes</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Together these inputs establish why Observation_Class alone is too coarse</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-    </row>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>and what the structural differences are within the Findings class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PURPOSE</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Analysis output combining domain metadata with our structural categorization</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-    </row>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>and COSMoS coverage counts. Evolves as we refine the categorization or COSMoS updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SHEETS</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Domain_Analysis</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>One row per domain — structural type + behavioural group + COSMoS coverage (56 rows)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-    </row>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Structural_Types</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Definition of each Structural_Type value (10 rows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>COLUMN DESCRIPTIONS — Domain_Analysis</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Two-letter SDTM domain abbreviation (join key to SDTM_Domain_Metadata.xlsx)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Domain_Name</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Full domain name (carried from metadata for readability)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Observation_Class</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SDTM observation class (carried from metadata for readability)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Structural_Type</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Our categorization — see Structural_Types sheet</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>Behavioural_Group</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>COSMoS-empirical behavioural classification (31 domains with COSMoS content; blank for others). See COSMoS_Domain_Pattern_Inventory.xlsx for group definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>COSMoS_BCs</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Count of unique Biomedical Concepts with DSSs in this domain (0 = no coverage)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-    </row>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>COSMoS_DSSs</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Count of Dataset Specializations in this domain (0 = no coverage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>SDTM Domain Analysis</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>COLUMN DESCRIPTIONS — Structural_Types</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="2" t="n"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Structural_Type</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Type name used in the Domain_Analysis sheet</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n"/>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>What this type represents</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Base data</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>SDTM_Domain_Metadata.xlsx (this track, machine_actionable/)</t>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Key_Characteristics</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Architectural properties that distinguish this type</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>CT analysis</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>sdtm-ct-analysis skill — 1,181 codelists, 25 categories</t>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>COSMoS_Pattern</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>How BCs and DSSs relate in domains of this type</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>COSMoS data</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>COSMoS_BC_DSS.xlsx from cosmos-bc-dss track</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Created</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-    </row>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Example_Domains</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Representative domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Repository</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/kerfors/cdisc-for-ai</t>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>COVERAGE STATISTICS</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr"/>
-      <c r="B57" s="2" t="n"/>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Total domains</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>INPUTS</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n"/>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>With COSMoS coverage</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>The Structural_Type categorization is derived from two analytical inputs:</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n"/>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Without COSMoS coverage</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
-      <c r="B60" s="2" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>1. SDTM CT Category Discovery</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n"/>
-    </row>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Total COSMoS DSSs</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1123</t>
+        </is>
+      </c>
+    </row>
+    <row r="61"/>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Assignments</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>skills/sdtm-ct-analysis/example-output/SDTM_CT_Category_Discovery_assignments.csv</t>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DESIGN DECISIONS</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Profiles</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>skills/sdtm-ct-analysis/example-output/SDTM_CT_Category_Profiles.md</t>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Structural_Type does not exist in any CDISC publication. It is our contribution,</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Key finding</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>25 categories; 83% of codelists (976/1181) are instrument-specific;</t>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>based on how domain data is architecturally structured and consumed. It cross-cuts</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr"/>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>extensibility flag separates 56 domain-level from 353 instrument-specific test code codelists</t>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SDTM's Observation_Class with usage patterns derived from the CT category analysis</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr"/>
-      <c r="B66" s="2" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>2. COSMoS BC/DSS content analysis</t>
-        </is>
-      </c>
-    </row>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>and COSMoS content inspection listed under INPUTS above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67"/>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Interim file</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>cosmos-bc-dss/interim/COSMoS_BC_DSS.xlsx</t>
+      <c r="A68" s="26" t="inlineStr">
+        <is>
+          <t>Behavioural_Group is a COSMoS-empirical classification that refines Structural_Type</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Content doc</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>cosmos-bc-dss/docs/COSMoS_Content_and_QC.md</t>
+      <c r="A69" s="26" t="inlineStr">
+        <is>
+          <t>where observed BC→DSS patterns diverge from IG-level expectations.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Key finding</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>BC-&gt;DSS decomposition by specimen/method only occurs in specimen-based domains;</t>
+      <c r="A70" s="26" t="inlineStr">
+        <is>
+          <t>Key divergence: "Specimen-based Findings" splits into Specimen Findings, Immunogenicity</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>instrument domains are 1:1 (DSS=BC); BC hierarchy provides instrument-&gt;question grouping</t>
+      <c r="A71" s="26" t="inlineStr">
+        <is>
+          <t>Findings, and Genomics Findings. UR reclassified to Domain-specific Findings.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Domain_Name and Observation_Class are carried from the metadata file for readability.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Together these inputs establish why Observation_Class alone is too coarse</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>and what the structural differences are within the Findings class.</t>
-        </is>
-      </c>
-    </row>
+          <t>The authoritative source for those columns is SDTM_Domain_Metadata.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74"/>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>PURPOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Analysis output combining domain metadata with our structural categorization</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>and COSMoS coverage counts. Evolves as we refine the categorization or COSMoS updates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>SHEETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Domain_Analysis</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>One row per domain — structural type + COSMoS coverage (56 rows)</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Structural_Types</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Definition of each Structural_Type value (10 rows)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>COLUMN DESCRIPTIONS — Domain_Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Two-letter SDTM domain abbreviation (join key to SDTM_Domain_Metadata.xlsx)</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Domain_Name</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Full domain name (carried from metadata for readability)</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Observation_Class</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>SDTM observation class (carried from metadata for readability)</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Structural_Type</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Our categorization — see Structural_Types sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>COSMoS_BCs</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Count of unique Biomedical Concepts with DSSs in this domain (0 = no coverage)</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>COSMoS_DSSs</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Count of Dataset Specializations in this domain (0 = no coverage)</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>COLUMN DESCRIPTIONS — Structural_Types</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Structural_Type</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Type name used in the Domain_Analysis sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>What this type represents</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Key_Characteristics</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Architectural properties that distinguish this type</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>COSMoS_Pattern</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>How BCs and DSSs relate in domains of this type</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Example_Domains</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Representative domains</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>COVERAGE STATISTICS</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Total domains</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>With COSMoS coverage</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Without COSMoS coverage</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Total COSMoS DSSs</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>1123</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>DESIGN DECISIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Structural_Type does not exist in any CDISC publication. It is our contribution,</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>based on how domain data is architecturally structured and consumed. It cross-cuts</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>SDTM's Observation_Class with usage patterns derived from the CT category analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>and COSMoS content inspection listed under INPUTS above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Domain_Name and Observation_Class are carried from the metadata file for readability.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>The authoritative source for those columns is SDTM_Domain_Metadata.xlsx.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>COSMoS coverage counts are point-in-time (March 2026). COSMoS is actively evolving.</t>
         </is>
@@ -1341,14 +1230,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1373,12 +1262,17 @@
           <t>Structural_Type</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>Behavioural_Group</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
         <is>
           <t>COSMoS_BCs</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="28" t="inlineStr">
         <is>
           <t>COSMoS_DSSs</t>
         </is>
@@ -1405,10 +1299,11 @@
           <t>Special-Purpose</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1433,12 +1328,17 @@
           <t>Special-Purpose</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n">
-        <v>5</v>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Special-Purpose</t>
+        </is>
       </c>
       <c r="F3" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="G3" s="5" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1461,10 +1361,11 @@
           <t>Special-Purpose</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1489,10 +1390,11 @@
           <t>Special-Purpose</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1517,10 +1419,11 @@
           <t>Special-Purpose</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1545,10 +1448,11 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1573,10 +1477,15 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Interventions</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="G8" s="5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1601,10 +1510,15 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Interventions</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="G9" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1629,12 +1543,17 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>1</v>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Interventions</t>
+        </is>
       </c>
       <c r="F10" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="G10" s="5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1657,10 +1576,11 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1685,10 +1605,15 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Interventions</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="G12" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1713,10 +1638,15 @@
           <t>Interventions</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Interventions</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="G13" s="5" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1741,10 +1671,15 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="G14" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1769,12 +1704,17 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>7</v>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
       </c>
       <c r="F15" s="5" t="n">
         <v>7</v>
       </c>
+      <c r="G15" s="5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1797,10 +1737,11 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1825,12 +1766,17 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>18</v>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
       </c>
       <c r="F17" s="5" t="n">
         <v>18</v>
       </c>
+      <c r="G17" s="5" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1853,10 +1799,11 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1881,10 +1828,11 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E19" s="2" t="n"/>
       <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1909,10 +1857,15 @@
           <t>Events</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="G20" s="5" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1937,10 +1890,11 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E21" s="2" t="n"/>
       <c r="F21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1965,12 +1919,17 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E22" s="5" t="n">
-        <v>13</v>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Domain-specific Findings</t>
+        </is>
       </c>
       <c r="F22" s="5" t="n">
         <v>13</v>
       </c>
+      <c r="G22" s="5" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1993,12 +1952,17 @@
           <t>Measurement Findings</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n">
-        <v>33</v>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Measurement Findings</t>
+        </is>
       </c>
       <c r="F23" s="5" t="n">
         <v>33</v>
       </c>
+      <c r="G23" s="5" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2021,12 +1985,17 @@
           <t>Clinical Assessment Findings</t>
         </is>
       </c>
-      <c r="E24" s="5" t="n">
-        <v>2</v>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Assessment</t>
+        </is>
       </c>
       <c r="F24" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="G24" s="5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2049,10 +2018,11 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E25" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2077,10 +2047,11 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E26" s="2" t="n"/>
       <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2105,10 +2076,15 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Genomics Findings</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="G27" s="5" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2133,10 +2109,15 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Immunogenicity Findings</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="G28" s="5" t="n">
         <v>290</v>
       </c>
     </row>
@@ -2161,10 +2142,15 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Specimen Findings</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="G29" s="5" t="n">
         <v>142</v>
       </c>
     </row>
@@ -2189,10 +2175,15 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Specimen Findings</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="G30" s="5" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2217,10 +2208,15 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Specimen Findings</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="G31" s="5" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2245,10 +2241,11 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E32" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E32" s="2" t="n"/>
       <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2273,10 +2270,11 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E33" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E33" s="2" t="n"/>
       <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2301,10 +2299,11 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E34" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2329,12 +2328,17 @@
           <t>Clinical Assessment Findings</t>
         </is>
       </c>
-      <c r="E35" s="5" t="n">
-        <v>12</v>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Assessment</t>
+        </is>
       </c>
       <c r="F35" s="5" t="n">
         <v>12</v>
       </c>
+      <c r="G35" s="5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -2357,12 +2361,17 @@
           <t>Instrument Findings</t>
         </is>
       </c>
-      <c r="E36" s="5" t="n">
-        <v>23</v>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Instrument Findings</t>
+        </is>
       </c>
       <c r="F36" s="5" t="n">
         <v>23</v>
       </c>
+      <c r="G36" s="5" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -2385,10 +2394,15 @@
           <t>Measurement Findings</t>
         </is>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Measurement Findings</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="G37" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2413,12 +2427,17 @@
           <t>Instrument Findings</t>
         </is>
       </c>
-      <c r="E38" s="5" t="n">
-        <v>17</v>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Instrument Findings</t>
+        </is>
       </c>
       <c r="F38" s="5" t="n">
         <v>17</v>
       </c>
+      <c r="G38" s="5" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2441,12 +2460,17 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E39" s="5" t="n">
-        <v>96</v>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Domain-specific Findings</t>
+        </is>
       </c>
       <c r="F39" s="5" t="n">
         <v>96</v>
       </c>
+      <c r="G39" s="5" t="n">
+        <v>96</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2469,10 +2493,15 @@
           <t>Instrument Findings</t>
         </is>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Instrument Findings</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
         <v>129</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="G40" s="5" t="n">
         <v>135</v>
       </c>
     </row>
@@ -2497,12 +2526,17 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E41" s="5" t="n">
-        <v>2</v>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Domain-specific Findings</t>
+        </is>
       </c>
       <c r="F41" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="G41" s="5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2525,12 +2559,17 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E42" s="5" t="n">
-        <v>12</v>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Domain-specific Findings</t>
+        </is>
       </c>
       <c r="F42" s="5" t="n">
         <v>12</v>
       </c>
+      <c r="G42" s="5" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2553,10 +2592,11 @@
           <t>Domain-specific Findings</t>
         </is>
       </c>
-      <c r="E43" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E43" s="2" t="n"/>
       <c r="F43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2581,10 +2621,15 @@
           <t>Clinical Assessment Findings</t>
         </is>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Assessment</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="G44" s="5" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2609,10 +2654,15 @@
           <t>Clinical Assessment Findings</t>
         </is>
       </c>
-      <c r="E45" s="5" t="n">
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Assessment</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="G45" s="5" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2637,12 +2687,17 @@
           <t>Specimen-based Findings</t>
         </is>
       </c>
-      <c r="E46" s="5" t="n">
-        <v>10</v>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Domain-specific Findings</t>
+        </is>
       </c>
       <c r="F46" s="5" t="n">
         <v>10</v>
       </c>
+      <c r="G46" s="5" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2665,10 +2720,15 @@
           <t>Measurement Findings</t>
         </is>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Measurement Findings</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="G47" s="5" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2693,10 +2753,11 @@
           <t>Measurement Findings</t>
         </is>
       </c>
-      <c r="E48" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E48" s="2" t="n"/>
       <c r="F48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2721,10 +2782,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E49" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E49" s="2" t="n"/>
       <c r="F49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2749,10 +2811,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E50" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E50" s="2" t="n"/>
       <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2777,10 +2840,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E51" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E51" s="2" t="n"/>
       <c r="F51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2805,10 +2869,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E52" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E52" s="2" t="n"/>
       <c r="F52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2833,10 +2898,15 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E53" s="5" t="n">
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Trial Design</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="n">
         <v>128</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="G53" s="5" t="n">
         <v>129</v>
       </c>
     </row>
@@ -2861,10 +2931,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E54" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E54" s="2" t="n"/>
       <c r="F54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2889,10 +2960,11 @@
           <t>Trial Design</t>
         </is>
       </c>
-      <c r="E55" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E55" s="2" t="n"/>
       <c r="F55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2917,10 +2989,11 @@
           <t>Relationship</t>
         </is>
       </c>
-      <c r="E56" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E56" s="2" t="n"/>
       <c r="F56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2945,10 +3018,11 @@
           <t>Relationship</t>
         </is>
       </c>
-      <c r="E57" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="E57" s="2" t="n"/>
       <c r="F57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>